<commit_message>
Rename ReadMe to README.md
</commit_message>
<xml_diff>
--- a/chrona-sample-timeline.xlsx
+++ b/chrona-sample-timeline.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline Data" sheetId="1" r:id="R907e66a3e1614aae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="2" r:id="Ra4004e2e0a144040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline Data" sheetId="1" r:id="Rb6b7396466c34d95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="2" r:id="R0a6e8ca36b8444fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -46,7 +46,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -77,11 +77,51 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -377,8 +417,8 @@
       <x:c r="I2" s="11" t="str">
         <x:v>The thirteen colonies declared independence from Great Britain.</x:v>
       </x:c>
-      <x:c r="J2" s="11" t="str"/>
-      <x:c r="K2" s="11" t="str"/>
+      <x:c r="J2" s="11"/>
+      <x:c r="K2" s="11"/>
       <x:c r="L2" s="11" t="str">
         <x:v>https://upload.wikimedia.org/wikipedia/commons/1/15/Declaration_independence.jpg</x:v>
       </x:c>
@@ -388,13 +428,11 @@
       <x:c r="N2" s="11" t="str">
         <x:v>Declaration of Independence</x:v>
       </x:c>
-      <x:c r="O2" s="11" t="str"/>
+      <x:c r="O2" s="11"/>
       <x:c r="P2" s="11" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="Q2" s="11" t="str">
-        <x:v>Event</x:v>
-      </x:c>
+      <x:c r="Q2" s="11"/>
       <x:c r="R2" s="11" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -427,8 +465,8 @@
       <x:c r="I3" s="11" t="str">
         <x:v>Delegates signed the Constitution in Philadelphia.</x:v>
       </x:c>
-      <x:c r="J3" s="11" t="str"/>
-      <x:c r="K3" s="11" t="str"/>
+      <x:c r="J3" s="11"/>
+      <x:c r="K3" s="11"/>
       <x:c r="L3" s="11" t="str">
         <x:v>https://upload.wikimedia.org/wikipedia/commons/4/4d/Scene_at_the_Signing_of_the_Constitution_of_the_United_States.jpg</x:v>
       </x:c>
@@ -438,13 +476,11 @@
       <x:c r="N3" s="11" t="str">
         <x:v>Signing of the U.S. Constitution</x:v>
       </x:c>
-      <x:c r="O3" s="11" t="str"/>
+      <x:c r="O3" s="11"/>
       <x:c r="P3" s="11" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="Q3" s="11" t="str">
-        <x:v>Event</x:v>
-      </x:c>
+      <x:c r="Q3" s="11"/>
       <x:c r="R3" s="11" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -475,8 +511,8 @@
       <x:c r="I4" s="11" t="str">
         <x:v>Conflict between Qing China and Britain led to the Treaty of Nanking.</x:v>
       </x:c>
-      <x:c r="J4" s="11" t="str"/>
-      <x:c r="K4" s="11" t="str"/>
+      <x:c r="J4" s="11"/>
+      <x:c r="K4" s="11"/>
       <x:c r="L4" s="11" t="str">
         <x:v>https://upload.wikimedia.org/wikipedia/commons/0/0e/Destroying_Chinese_war_junks%2C_by_E._Duncan_%281843%29.jpg</x:v>
       </x:c>
@@ -486,13 +522,11 @@
       <x:c r="N4" s="11" t="str">
         <x:v>Naval battle during the First Opium War</x:v>
       </x:c>
-      <x:c r="O4" s="11" t="str"/>
+      <x:c r="O4" s="11"/>
       <x:c r="P4" s="11" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="Q4" s="11" t="str">
-        <x:v>Event</x:v>
-      </x:c>
+      <x:c r="Q4" s="11"/>
       <x:c r="R4" s="11" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -531,8 +565,8 @@
       <x:c r="I5" s="11" t="str">
         <x:v>War between the Union and the Confederacy transformed the United States and ended legal slavery.</x:v>
       </x:c>
-      <x:c r="J5" s="11" t="str"/>
-      <x:c r="K5" s="11" t="str"/>
+      <x:c r="J5" s="11"/>
+      <x:c r="K5" s="11"/>
       <x:c r="L5" s="11" t="str">
         <x:v>https://upload.wikimedia.org/wikipedia/commons/9/9a/Fall_of_Richmond_Va_on_the_night_of_April_2nd_1865.jpg</x:v>
       </x:c>
@@ -542,13 +576,11 @@
       <x:c r="N5" s="11" t="str">
         <x:v>Richmond during the Civil War</x:v>
       </x:c>
-      <x:c r="O5" s="11" t="str"/>
+      <x:c r="O5" s="11"/>
       <x:c r="P5" s="11" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="Q5" s="11" t="str">
-        <x:v>Event</x:v>
-      </x:c>
+      <x:c r="Q5" s="11"/>
       <x:c r="R5" s="11" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -587,8 +619,8 @@
       <x:c r="I6" s="11" t="str">
         <x:v>The revolution ended imperial rule and led to the establishment of the Republic of China.</x:v>
       </x:c>
-      <x:c r="J6" s="11" t="str"/>
-      <x:c r="K6" s="11" t="str"/>
+      <x:c r="J6" s="11"/>
+      <x:c r="K6" s="11"/>
       <x:c r="L6" s="11" t="str">
         <x:v>https://upload.wikimedia.org/wikipedia/commons/8/8f/Wuchang_Uprising.jpg</x:v>
       </x:c>
@@ -598,13 +630,11 @@
       <x:c r="N6" s="11" t="str">
         <x:v>Wuchang Uprising</x:v>
       </x:c>
-      <x:c r="O6" s="11" t="str"/>
+      <x:c r="O6" s="11"/>
       <x:c r="P6" s="11" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="Q6" s="11" t="str">
-        <x:v>Event</x:v>
-      </x:c>
+      <x:c r="Q6" s="11"/>
       <x:c r="R6" s="11" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -637,8 +667,8 @@
       <x:c r="I7" s="11" t="str">
         <x:v>The stock-market collapse became a defining event of the Great Depression.</x:v>
       </x:c>
-      <x:c r="J7" s="11" t="str"/>
-      <x:c r="K7" s="11" t="str"/>
+      <x:c r="J7" s="11"/>
+      <x:c r="K7" s="11"/>
       <x:c r="L7" s="11" t="str">
         <x:v>https://upload.wikimedia.org/wikipedia/commons/4/4c/Crowd_outside_nyse.jpg</x:v>
       </x:c>
@@ -648,13 +678,11 @@
       <x:c r="N7" s="11" t="str">
         <x:v>Crowd outside the New York Stock Exchange</x:v>
       </x:c>
-      <x:c r="O7" s="11" t="str"/>
+      <x:c r="O7" s="11"/>
       <x:c r="P7" s="11" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="Q7" s="11" t="str">
-        <x:v>Event</x:v>
-      </x:c>
+      <x:c r="Q7" s="11"/>
       <x:c r="R7" s="11" t="str">
         <x:v>Medium</x:v>
       </x:c>
@@ -693,8 +721,8 @@
       <x:c r="I8" s="11" t="str">
         <x:v>Full-scale war between China and Japan became part of the wider Second World War.</x:v>
       </x:c>
-      <x:c r="J8" s="11" t="str"/>
-      <x:c r="K8" s="11" t="str"/>
+      <x:c r="J8" s="11"/>
+      <x:c r="K8" s="11"/>
       <x:c r="L8" s="11" t="str">
         <x:v>https://upload.wikimedia.org/wikipedia/commons/4/46/Chinese_soldiers_in_house_to_house_fighting_in_Tai%27er_zhuang.jpg</x:v>
       </x:c>
@@ -704,13 +732,11 @@
       <x:c r="N8" s="11" t="str">
         <x:v>Chinese soldiers during the war</x:v>
       </x:c>
-      <x:c r="O8" s="11" t="str"/>
+      <x:c r="O8" s="11"/>
       <x:c r="P8" s="11" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="Q8" s="11" t="str">
-        <x:v>Event</x:v>
-      </x:c>
+      <x:c r="Q8" s="11"/>
       <x:c r="R8" s="11" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -758,13 +784,11 @@
       <x:c r="N9" s="11" t="str">
         <x:v>Proclamation ceremony in Beijing</x:v>
       </x:c>
-      <x:c r="O9" s="11" t="str"/>
+      <x:c r="O9" s="11"/>
       <x:c r="P9" s="11" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="Q9" s="11" t="str">
-        <x:v>Event</x:v>
-      </x:c>
+      <x:c r="Q9" s="11"/>
       <x:c r="R9" s="11" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -812,13 +836,11 @@
       <x:c r="N10" s="11" t="str">
         <x:v>Buzz Aldrin on the Moon</x:v>
       </x:c>
-      <x:c r="O10" s="11" t="str"/>
+      <x:c r="O10" s="11"/>
       <x:c r="P10" s="11" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="Q10" s="11" t="str">
-        <x:v>Event</x:v>
-      </x:c>
+      <x:c r="Q10" s="11"/>
       <x:c r="R10" s="11" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -851,8 +873,8 @@
       <x:c r="I11" s="11" t="str">
         <x:v>The Third Plenum marked the beginning of major economic reform under Deng Xiaoping.</x:v>
       </x:c>
-      <x:c r="J11" s="11" t="str"/>
-      <x:c r="K11" s="11" t="str"/>
+      <x:c r="J11" s="11"/>
+      <x:c r="K11" s="11"/>
       <x:c r="L11" s="11" t="str">
         <x:v>https://upload.wikimedia.org/wikipedia/commons/5/5c/Deng_Xiaoping_1979.jpg</x:v>
       </x:c>
@@ -862,13 +884,11 @@
       <x:c r="N11" s="11" t="str">
         <x:v>Deng Xiaoping</x:v>
       </x:c>
-      <x:c r="O11" s="11" t="str"/>
+      <x:c r="O11" s="11"/>
       <x:c r="P11" s="11" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="Q11" s="11" t="str">
-        <x:v>Event</x:v>
-      </x:c>
+      <x:c r="Q11" s="11"/>
       <x:c r="R11" s="11" t="str">
         <x:v>Major</x:v>
       </x:c>
@@ -899,17 +919,17 @@
       <x:c r="I12" s="11" t="str">
         <x:v>Reference period spanning the Roman imperial era in the West.</x:v>
       </x:c>
-      <x:c r="J12" s="11" t="str"/>
-      <x:c r="K12" s="11" t="str"/>
+      <x:c r="J12" s="11"/>
+      <x:c r="K12" s="11"/>
       <x:c r="L12" s="11"/>
       <x:c r="M12" s="11"/>
       <x:c r="N12" s="11"/>
-      <x:c r="O12" s="11" t="str"/>
+      <x:c r="O12" s="11"/>
       <x:c r="P12" s="11" t="str">
         <x:v>Ancient Rome</x:v>
       </x:c>
       <x:c r="Q12" s="11" t="str">
-        <x:v>Period</x:v>
+        <x:v>period</x:v>
       </x:c>
       <x:c r="R12" s="11" t="str">
         <x:v>Major</x:v>
@@ -941,17 +961,17 @@
       <x:c r="I13" s="11" t="str">
         <x:v>A simplified reference span for Britain’s imperial period.</x:v>
       </x:c>
-      <x:c r="J13" s="11" t="str"/>
-      <x:c r="K13" s="11" t="str"/>
+      <x:c r="J13" s="11"/>
+      <x:c r="K13" s="11"/>
       <x:c r="L13" s="11"/>
       <x:c r="M13" s="11"/>
       <x:c r="N13" s="11"/>
-      <x:c r="O13" s="11" t="str"/>
+      <x:c r="O13" s="11"/>
       <x:c r="P13" s="11" t="str">
         <x:v>Britain</x:v>
       </x:c>
       <x:c r="Q13" s="11" t="str">
-        <x:v>Period</x:v>
+        <x:v>period</x:v>
       </x:c>
       <x:c r="R13" s="11" t="str">
         <x:v>Major</x:v>
@@ -983,17 +1003,17 @@
       <x:c r="I14" s="11" t="str">
         <x:v>Period during which Adolf Hitler and the Nazi Party ruled Germany.</x:v>
       </x:c>
-      <x:c r="J14" s="11" t="str"/>
-      <x:c r="K14" s="11" t="str"/>
+      <x:c r="J14" s="11"/>
+      <x:c r="K14" s="11"/>
       <x:c r="L14" s="11"/>
       <x:c r="M14" s="11"/>
       <x:c r="N14" s="11"/>
-      <x:c r="O14" s="11" t="str"/>
+      <x:c r="O14" s="11"/>
       <x:c r="P14" s="11" t="str">
         <x:v>Germany</x:v>
       </x:c>
       <x:c r="Q14" s="11" t="str">
-        <x:v>Period</x:v>
+        <x:v>period</x:v>
       </x:c>
       <x:c r="R14" s="11" t="str">
         <x:v>Major</x:v>
@@ -1034,12 +1054,12 @@
       <x:c r="L15" s="11"/>
       <x:c r="M15" s="11"/>
       <x:c r="N15" s="11"/>
-      <x:c r="O15" s="11" t="str"/>
+      <x:c r="O15" s="11"/>
       <x:c r="P15" s="11" t="str">
         <x:v>China</x:v>
       </x:c>
       <x:c r="Q15" s="11" t="str">
-        <x:v>Period</x:v>
+        <x:v>period</x:v>
       </x:c>
       <x:c r="R15" s="11" t="str">
         <x:v>Major</x:v>
@@ -1049,12 +1069,2092 @@
       </x:c>
       <x:c r="T15" s="11" t="str">
         <x:v>CN-1644-1912-QING</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="11" t="n">
+        <x:v>1903</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C16" s="11" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D16" s="11"/>
+      <x:c r="E16" s="11"/>
+      <x:c r="F16" s="11"/>
+      <x:c r="G16" s="11"/>
+      <x:c r="H16" s="11" t="str">
+        <x:v>Wright Brothers’ First Powered Flight</x:v>
+      </x:c>
+      <x:c r="I16" s="11" t="str">
+        <x:v>The Wright brothers achieved the first controlled, sustained powered flight.</x:v>
+      </x:c>
+      <x:c r="J16" s="11"/>
+      <x:c r="K16" s="11"/>
+      <x:c r="L16" s="11"/>
+      <x:c r="M16" s="11"/>
+      <x:c r="N16" s="11"/>
+      <x:c r="O16" s="11"/>
+      <x:c r="P16" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q16" s="11"/>
+      <x:c r="R16" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S16" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T16" s="11" t="str">
+        <x:v>US-1903-WRIGHT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="11" t="n">
+        <x:v>1913</x:v>
+      </x:c>
+      <x:c r="B17" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D17" s="11"/>
+      <x:c r="E17" s="11"/>
+      <x:c r="F17" s="11"/>
+      <x:c r="G17" s="11"/>
+      <x:c r="H17" s="11" t="str">
+        <x:v>Federal Reserve Act Signed</x:v>
+      </x:c>
+      <x:c r="I17" s="11" t="str">
+        <x:v>The act created the Federal Reserve System.</x:v>
+      </x:c>
+      <x:c r="J17" s="11"/>
+      <x:c r="K17" s="11"/>
+      <x:c r="L17" s="11"/>
+      <x:c r="M17" s="11"/>
+      <x:c r="N17" s="11"/>
+      <x:c r="O17" s="11"/>
+      <x:c r="P17" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q17" s="11"/>
+      <x:c r="R17" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S17" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T17" s="11" t="str">
+        <x:v>US-1913-FED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="11" t="n">
+        <x:v>1933</x:v>
+      </x:c>
+      <x:c r="B18" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C18" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D18" s="11"/>
+      <x:c r="E18" s="11"/>
+      <x:c r="F18" s="11"/>
+      <x:c r="G18" s="11"/>
+      <x:c r="H18" s="11" t="str">
+        <x:v>New Deal Begins</x:v>
+      </x:c>
+      <x:c r="I18" s="11" t="str">
+        <x:v>Franklin D. Roosevelt launched relief, recovery, and reform programs during the Great Depression.</x:v>
+      </x:c>
+      <x:c r="J18" s="11"/>
+      <x:c r="K18" s="11"/>
+      <x:c r="L18" s="11"/>
+      <x:c r="M18" s="11"/>
+      <x:c r="N18" s="11"/>
+      <x:c r="O18" s="11"/>
+      <x:c r="P18" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q18" s="11"/>
+      <x:c r="R18" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S18" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T18" s="11" t="str">
+        <x:v>US-1933-NEW-DEAL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="11" t="n">
+        <x:v>1935</x:v>
+      </x:c>
+      <x:c r="B19" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C19" s="11" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D19" s="11"/>
+      <x:c r="E19" s="11"/>
+      <x:c r="F19" s="11"/>
+      <x:c r="G19" s="11"/>
+      <x:c r="H19" s="11" t="str">
+        <x:v>Social Security Act Signed</x:v>
+      </x:c>
+      <x:c r="I19" s="11" t="str">
+        <x:v>The act established federal old-age benefits and other social protections.</x:v>
+      </x:c>
+      <x:c r="J19" s="11"/>
+      <x:c r="K19" s="11"/>
+      <x:c r="L19" s="11"/>
+      <x:c r="M19" s="11"/>
+      <x:c r="N19" s="11"/>
+      <x:c r="O19" s="11"/>
+      <x:c r="P19" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q19" s="11"/>
+      <x:c r="R19" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S19" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T19" s="11" t="str">
+        <x:v>US-1935-SOCIAL-SECURITY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="11" t="n">
+        <x:v>1945</x:v>
+      </x:c>
+      <x:c r="B20" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C20" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D20" s="11"/>
+      <x:c r="E20" s="11"/>
+      <x:c r="F20" s="11"/>
+      <x:c r="G20" s="11"/>
+      <x:c r="H20" s="11" t="str">
+        <x:v>Atomic Bomb Dropped on Hiroshima</x:v>
+      </x:c>
+      <x:c r="I20" s="11" t="str">
+        <x:v>The United States used an atomic bomb on Hiroshima, opening the nuclear age.</x:v>
+      </x:c>
+      <x:c r="J20" s="11"/>
+      <x:c r="K20" s="11"/>
+      <x:c r="L20" s="11"/>
+      <x:c r="M20" s="11"/>
+      <x:c r="N20" s="11"/>
+      <x:c r="O20" s="11"/>
+      <x:c r="P20" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q20" s="11"/>
+      <x:c r="R20" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S20" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T20" s="11" t="str">
+        <x:v>US-1945-HIROSHIMA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="11" t="n">
+        <x:v>1956</x:v>
+      </x:c>
+      <x:c r="B21" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C21" s="11" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D21" s="11"/>
+      <x:c r="E21" s="11"/>
+      <x:c r="F21" s="11"/>
+      <x:c r="G21" s="11"/>
+      <x:c r="H21" s="11" t="str">
+        <x:v>Interstate Highway Act Signed</x:v>
+      </x:c>
+      <x:c r="I21" s="11" t="str">
+        <x:v>The act authorized the Interstate Highway System.</x:v>
+      </x:c>
+      <x:c r="J21" s="11"/>
+      <x:c r="K21" s="11"/>
+      <x:c r="L21" s="11"/>
+      <x:c r="M21" s="11"/>
+      <x:c r="N21" s="11"/>
+      <x:c r="O21" s="11"/>
+      <x:c r="P21" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q21" s="11"/>
+      <x:c r="R21" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S21" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T21" s="11" t="str">
+        <x:v>US-1956-INTERSTATE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="11" t="n">
+        <x:v>1964</x:v>
+      </x:c>
+      <x:c r="B22" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C22" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D22" s="11"/>
+      <x:c r="E22" s="11"/>
+      <x:c r="F22" s="11"/>
+      <x:c r="G22" s="11"/>
+      <x:c r="H22" s="11" t="str">
+        <x:v>Civil Rights Act Signed</x:v>
+      </x:c>
+      <x:c r="I22" s="11" t="str">
+        <x:v>The law outlawed major forms of discrimination and segregation.</x:v>
+      </x:c>
+      <x:c r="J22" s="11"/>
+      <x:c r="K22" s="11"/>
+      <x:c r="L22" s="11"/>
+      <x:c r="M22" s="11"/>
+      <x:c r="N22" s="11"/>
+      <x:c r="O22" s="11"/>
+      <x:c r="P22" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q22" s="11"/>
+      <x:c r="R22" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S22" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T22" s="11" t="str">
+        <x:v>US-1964-CIVIL-RIGHTS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="11" t="n">
+        <x:v>1965</x:v>
+      </x:c>
+      <x:c r="B23" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C23" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D23" s="11"/>
+      <x:c r="E23" s="11"/>
+      <x:c r="F23" s="11"/>
+      <x:c r="G23" s="11"/>
+      <x:c r="H23" s="11" t="str">
+        <x:v>Voting Rights Act Signed</x:v>
+      </x:c>
+      <x:c r="I23" s="11" t="str">
+        <x:v>The law strengthened federal protection against racial discrimination in voting.</x:v>
+      </x:c>
+      <x:c r="J23" s="11"/>
+      <x:c r="K23" s="11"/>
+      <x:c r="L23" s="11"/>
+      <x:c r="M23" s="11"/>
+      <x:c r="N23" s="11"/>
+      <x:c r="O23" s="11"/>
+      <x:c r="P23" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q23" s="11"/>
+      <x:c r="R23" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S23" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T23" s="11" t="str">
+        <x:v>US-1965-VOTING-RIGHTS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="11" t="n">
+        <x:v>1974</x:v>
+      </x:c>
+      <x:c r="B24" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C24" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D24" s="11"/>
+      <x:c r="E24" s="11"/>
+      <x:c r="F24" s="11"/>
+      <x:c r="G24" s="11"/>
+      <x:c r="H24" s="11" t="str">
+        <x:v>Richard Nixon Resigns</x:v>
+      </x:c>
+      <x:c r="I24" s="11" t="str">
+        <x:v>Nixon became the first U.S. president to resign.</x:v>
+      </x:c>
+      <x:c r="J24" s="11"/>
+      <x:c r="K24" s="11"/>
+      <x:c r="L24" s="11"/>
+      <x:c r="M24" s="11"/>
+      <x:c r="N24" s="11"/>
+      <x:c r="O24" s="11"/>
+      <x:c r="P24" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q24" s="11"/>
+      <x:c r="R24" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S24" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T24" s="11" t="str">
+        <x:v>US-1974-NIXON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="11" t="n">
+        <x:v>1986</x:v>
+      </x:c>
+      <x:c r="B25" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C25" s="11" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D25" s="11"/>
+      <x:c r="E25" s="11"/>
+      <x:c r="F25" s="11"/>
+      <x:c r="G25" s="11"/>
+      <x:c r="H25" s="11" t="str">
+        <x:v>Space Shuttle Challenger Disaster</x:v>
+      </x:c>
+      <x:c r="I25" s="11" t="str">
+        <x:v>Challenger broke apart shortly after launch, killing all seven crew members.</x:v>
+      </x:c>
+      <x:c r="J25" s="11"/>
+      <x:c r="K25" s="11"/>
+      <x:c r="L25" s="11"/>
+      <x:c r="M25" s="11"/>
+      <x:c r="N25" s="11"/>
+      <x:c r="O25" s="11"/>
+      <x:c r="P25" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q25" s="11"/>
+      <x:c r="R25" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S25" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T25" s="11" t="str">
+        <x:v>US-1986-CHALLENGER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="11" t="n">
+        <x:v>1991</x:v>
+      </x:c>
+      <x:c r="B26" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C26" s="11" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D26" s="11"/>
+      <x:c r="E26" s="11"/>
+      <x:c r="F26" s="11"/>
+      <x:c r="G26" s="11"/>
+      <x:c r="H26" s="11" t="str">
+        <x:v>Operation Desert Storm Begins</x:v>
+      </x:c>
+      <x:c r="I26" s="11" t="str">
+        <x:v>A U.S.-led coalition began a campaign to expel Iraqi forces from Kuwait.</x:v>
+      </x:c>
+      <x:c r="J26" s="11"/>
+      <x:c r="K26" s="11"/>
+      <x:c r="L26" s="11"/>
+      <x:c r="M26" s="11"/>
+      <x:c r="N26" s="11"/>
+      <x:c r="O26" s="11"/>
+      <x:c r="P26" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q26" s="11"/>
+      <x:c r="R26" s="11" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="S26" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T26" s="11" t="str">
+        <x:v>US-1991-DESERT-STORM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="11" t="n">
+        <x:v>2010</x:v>
+      </x:c>
+      <x:c r="B27" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C27" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D27" s="11"/>
+      <x:c r="E27" s="11"/>
+      <x:c r="F27" s="11"/>
+      <x:c r="G27" s="11"/>
+      <x:c r="H27" s="11" t="str">
+        <x:v>Affordable Care Act Signed</x:v>
+      </x:c>
+      <x:c r="I27" s="11" t="str">
+        <x:v>The law expanded health-insurance coverage and changed the U.S. healthcare system.</x:v>
+      </x:c>
+      <x:c r="J27" s="11"/>
+      <x:c r="K27" s="11"/>
+      <x:c r="L27" s="11"/>
+      <x:c r="M27" s="11"/>
+      <x:c r="N27" s="11"/>
+      <x:c r="O27" s="11"/>
+      <x:c r="P27" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q27" s="11"/>
+      <x:c r="R27" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S27" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T27" s="11" t="str">
+        <x:v>US-2010-ACA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="11" t="n">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="B28" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C28" s="11" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="D28" s="11"/>
+      <x:c r="E28" s="11"/>
+      <x:c r="F28" s="11"/>
+      <x:c r="G28" s="11"/>
+      <x:c r="H28" s="11" t="str">
+        <x:v>Same-Sex Marriage Legalized Nationwide</x:v>
+      </x:c>
+      <x:c r="I28" s="11" t="str">
+        <x:v>The Supreme Court recognized a constitutional right for same-sex couples to marry.</x:v>
+      </x:c>
+      <x:c r="J28" s="11"/>
+      <x:c r="K28" s="11"/>
+      <x:c r="L28" s="11"/>
+      <x:c r="M28" s="11"/>
+      <x:c r="N28" s="11"/>
+      <x:c r="O28" s="11"/>
+      <x:c r="P28" s="11" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="Q28" s="11"/>
+      <x:c r="R28" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S28" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T28" s="11" t="str">
+        <x:v>US-2015-OBERGEFELL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="11" t="n">
+        <x:v>1901</x:v>
+      </x:c>
+      <x:c r="B29" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C29" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="D29" s="11"/>
+      <x:c r="E29" s="11"/>
+      <x:c r="F29" s="11"/>
+      <x:c r="G29" s="11"/>
+      <x:c r="H29" s="11" t="str">
+        <x:v>Queen Victoria Dies</x:v>
+      </x:c>
+      <x:c r="I29" s="11" t="str">
+        <x:v>Victoria’s death ended the Victorian era and brought Edward VII to the throne.</x:v>
+      </x:c>
+      <x:c r="J29" s="11"/>
+      <x:c r="K29" s="11"/>
+      <x:c r="L29" s="11"/>
+      <x:c r="M29" s="11"/>
+      <x:c r="N29" s="11"/>
+      <x:c r="O29" s="11"/>
+      <x:c r="P29" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q29" s="11"/>
+      <x:c r="R29" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S29" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T29" s="11" t="str">
+        <x:v>GB-1901-VICTORIA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="11" t="n">
+        <x:v>1918</x:v>
+      </x:c>
+      <x:c r="B30" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C30" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D30" s="11"/>
+      <x:c r="E30" s="11"/>
+      <x:c r="F30" s="11"/>
+      <x:c r="G30" s="11"/>
+      <x:c r="H30" s="11" t="str">
+        <x:v>Representation of the People Act</x:v>
+      </x:c>
+      <x:c r="I30" s="11" t="str">
+        <x:v>The act greatly expanded voting rights, including for many women over age 30.</x:v>
+      </x:c>
+      <x:c r="J30" s="11"/>
+      <x:c r="K30" s="11"/>
+      <x:c r="L30" s="11"/>
+      <x:c r="M30" s="11"/>
+      <x:c r="N30" s="11"/>
+      <x:c r="O30" s="11"/>
+      <x:c r="P30" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q30" s="11"/>
+      <x:c r="R30" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S30" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T30" s="11" t="str">
+        <x:v>GB-1918-VOTING</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="11" t="n">
+        <x:v>1922</x:v>
+      </x:c>
+      <x:c r="B31" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C31" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D31" s="11"/>
+      <x:c r="E31" s="11"/>
+      <x:c r="F31" s="11"/>
+      <x:c r="G31" s="11"/>
+      <x:c r="H31" s="11" t="str">
+        <x:v>BBC Founded</x:v>
+      </x:c>
+      <x:c r="I31" s="11" t="str">
+        <x:v>The British Broadcasting Company was formed.</x:v>
+      </x:c>
+      <x:c r="J31" s="11"/>
+      <x:c r="K31" s="11"/>
+      <x:c r="L31" s="11"/>
+      <x:c r="M31" s="11"/>
+      <x:c r="N31" s="11"/>
+      <x:c r="O31" s="11"/>
+      <x:c r="P31" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q31" s="11"/>
+      <x:c r="R31" s="11" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="S31" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T31" s="11" t="str">
+        <x:v>GB-1922-BBC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="11" t="n">
+        <x:v>1926</x:v>
+      </x:c>
+      <x:c r="B32" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C32" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D32" s="11"/>
+      <x:c r="E32" s="11"/>
+      <x:c r="F32" s="11"/>
+      <x:c r="G32" s="11"/>
+      <x:c r="H32" s="11" t="str">
+        <x:v>General Strike Begins</x:v>
+      </x:c>
+      <x:c r="I32" s="11" t="str">
+        <x:v>Millions of workers joined Britain’s General Strike.</x:v>
+      </x:c>
+      <x:c r="J32" s="11"/>
+      <x:c r="K32" s="11"/>
+      <x:c r="L32" s="11"/>
+      <x:c r="M32" s="11"/>
+      <x:c r="N32" s="11"/>
+      <x:c r="O32" s="11"/>
+      <x:c r="P32" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q32" s="11"/>
+      <x:c r="R32" s="11" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="S32" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T32" s="11" t="str">
+        <x:v>GB-1926-STRIKE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="11" t="n">
+        <x:v>1936</x:v>
+      </x:c>
+      <x:c r="B33" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C33" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D33" s="11"/>
+      <x:c r="E33" s="11"/>
+      <x:c r="F33" s="11"/>
+      <x:c r="G33" s="11"/>
+      <x:c r="H33" s="11" t="str">
+        <x:v>Edward VIII Abdicates</x:v>
+      </x:c>
+      <x:c r="I33" s="11" t="str">
+        <x:v>Edward VIII gave up the throne to marry Wallis Simpson.</x:v>
+      </x:c>
+      <x:c r="J33" s="11"/>
+      <x:c r="K33" s="11"/>
+      <x:c r="L33" s="11"/>
+      <x:c r="M33" s="11"/>
+      <x:c r="N33" s="11"/>
+      <x:c r="O33" s="11"/>
+      <x:c r="P33" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q33" s="11"/>
+      <x:c r="R33" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S33" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T33" s="11" t="str">
+        <x:v>GB-1936-ABDICATION</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="11" t="n">
+        <x:v>1940</x:v>
+      </x:c>
+      <x:c r="B34" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C34" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D34" s="11"/>
+      <x:c r="E34" s="11"/>
+      <x:c r="F34" s="11"/>
+      <x:c r="G34" s="11"/>
+      <x:c r="H34" s="11" t="str">
+        <x:v>Battle of Britain Begins</x:v>
+      </x:c>
+      <x:c r="I34" s="11" t="str">
+        <x:v>The Royal Air Force fought Germany’s Luftwaffe over Britain.</x:v>
+      </x:c>
+      <x:c r="J34" s="11"/>
+      <x:c r="K34" s="11"/>
+      <x:c r="L34" s="11"/>
+      <x:c r="M34" s="11"/>
+      <x:c r="N34" s="11"/>
+      <x:c r="O34" s="11"/>
+      <x:c r="P34" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q34" s="11"/>
+      <x:c r="R34" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S34" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T34" s="11" t="str">
+        <x:v>GB-1940-BATTLE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="11" t="n">
+        <x:v>1948</x:v>
+      </x:c>
+      <x:c r="B35" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C35" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D35" s="11"/>
+      <x:c r="E35" s="11"/>
+      <x:c r="F35" s="11"/>
+      <x:c r="G35" s="11"/>
+      <x:c r="H35" s="11" t="str">
+        <x:v>National Health Service Launches</x:v>
+      </x:c>
+      <x:c r="I35" s="11" t="str">
+        <x:v>The NHS began providing publicly funded healthcare.</x:v>
+      </x:c>
+      <x:c r="J35" s="11"/>
+      <x:c r="K35" s="11"/>
+      <x:c r="L35" s="11"/>
+      <x:c r="M35" s="11"/>
+      <x:c r="N35" s="11"/>
+      <x:c r="O35" s="11"/>
+      <x:c r="P35" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q35" s="11"/>
+      <x:c r="R35" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S35" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T35" s="11" t="str">
+        <x:v>GB-1948-NHS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="11" t="n">
+        <x:v>1952</x:v>
+      </x:c>
+      <x:c r="B36" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C36" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D36" s="11"/>
+      <x:c r="E36" s="11"/>
+      <x:c r="F36" s="11"/>
+      <x:c r="G36" s="11"/>
+      <x:c r="H36" s="11" t="str">
+        <x:v>Elizabeth II Becomes Queen</x:v>
+      </x:c>
+      <x:c r="I36" s="11" t="str">
+        <x:v>Elizabeth II acceded to the throne after George VI died.</x:v>
+      </x:c>
+      <x:c r="J36" s="11"/>
+      <x:c r="K36" s="11"/>
+      <x:c r="L36" s="11"/>
+      <x:c r="M36" s="11"/>
+      <x:c r="N36" s="11"/>
+      <x:c r="O36" s="11"/>
+      <x:c r="P36" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q36" s="11"/>
+      <x:c r="R36" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S36" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T36" s="11" t="str">
+        <x:v>GB-1952-ELIZABETH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="11" t="n">
+        <x:v>1956</x:v>
+      </x:c>
+      <x:c r="B37" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C37" s="11" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D37" s="11"/>
+      <x:c r="E37" s="11"/>
+      <x:c r="F37" s="11"/>
+      <x:c r="G37" s="11"/>
+      <x:c r="H37" s="11" t="str">
+        <x:v>Suez Crisis Begins</x:v>
+      </x:c>
+      <x:c r="I37" s="11" t="str">
+        <x:v>The Suez Crisis exposed Britain’s reduced global power.</x:v>
+      </x:c>
+      <x:c r="J37" s="11"/>
+      <x:c r="K37" s="11"/>
+      <x:c r="L37" s="11"/>
+      <x:c r="M37" s="11"/>
+      <x:c r="N37" s="11"/>
+      <x:c r="O37" s="11"/>
+      <x:c r="P37" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q37" s="11"/>
+      <x:c r="R37" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S37" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T37" s="11" t="str">
+        <x:v>GB-1956-SUEZ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="11" t="n">
+        <x:v>1973</x:v>
+      </x:c>
+      <x:c r="B38" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C38" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D38" s="11"/>
+      <x:c r="E38" s="11"/>
+      <x:c r="F38" s="11"/>
+      <x:c r="G38" s="11"/>
+      <x:c r="H38" s="11" t="str">
+        <x:v>United Kingdom Joins the EEC</x:v>
+      </x:c>
+      <x:c r="I38" s="11" t="str">
+        <x:v>The United Kingdom entered the European Economic Community.</x:v>
+      </x:c>
+      <x:c r="J38" s="11"/>
+      <x:c r="K38" s="11"/>
+      <x:c r="L38" s="11"/>
+      <x:c r="M38" s="11"/>
+      <x:c r="N38" s="11"/>
+      <x:c r="O38" s="11"/>
+      <x:c r="P38" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q38" s="11"/>
+      <x:c r="R38" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S38" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T38" s="11" t="str">
+        <x:v>GB-1973-EEC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="11" t="n">
+        <x:v>1979</x:v>
+      </x:c>
+      <x:c r="B39" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C39" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D39" s="11"/>
+      <x:c r="E39" s="11"/>
+      <x:c r="F39" s="11"/>
+      <x:c r="G39" s="11"/>
+      <x:c r="H39" s="11" t="str">
+        <x:v>Margaret Thatcher Becomes Prime Minister</x:v>
+      </x:c>
+      <x:c r="I39" s="11" t="str">
+        <x:v>Thatcher became Britain’s first woman prime minister.</x:v>
+      </x:c>
+      <x:c r="J39" s="11"/>
+      <x:c r="K39" s="11"/>
+      <x:c r="L39" s="11"/>
+      <x:c r="M39" s="11"/>
+      <x:c r="N39" s="11"/>
+      <x:c r="O39" s="11"/>
+      <x:c r="P39" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q39" s="11"/>
+      <x:c r="R39" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S39" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T39" s="11" t="str">
+        <x:v>GB-1979-THATCHER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="11" t="n">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="B40" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C40" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D40" s="11"/>
+      <x:c r="E40" s="11"/>
+      <x:c r="F40" s="11"/>
+      <x:c r="G40" s="11"/>
+      <x:c r="H40" s="11" t="str">
+        <x:v>Brexit Referendum</x:v>
+      </x:c>
+      <x:c r="I40" s="11" t="str">
+        <x:v>UK voters chose to leave the European Union.</x:v>
+      </x:c>
+      <x:c r="J40" s="11"/>
+      <x:c r="K40" s="11"/>
+      <x:c r="L40" s="11"/>
+      <x:c r="M40" s="11"/>
+      <x:c r="N40" s="11"/>
+      <x:c r="O40" s="11"/>
+      <x:c r="P40" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q40" s="11"/>
+      <x:c r="R40" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S40" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T40" s="11" t="str">
+        <x:v>GB-2016-BREXIT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="11" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="B41" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C41" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D41" s="11"/>
+      <x:c r="E41" s="11"/>
+      <x:c r="F41" s="11"/>
+      <x:c r="G41" s="11"/>
+      <x:c r="H41" s="11" t="str">
+        <x:v>Queen Elizabeth II Dies</x:v>
+      </x:c>
+      <x:c r="I41" s="11" t="str">
+        <x:v>Elizabeth II died after a 70-year reign; Charles III became king.</x:v>
+      </x:c>
+      <x:c r="J41" s="11"/>
+      <x:c r="K41" s="11"/>
+      <x:c r="L41" s="11"/>
+      <x:c r="M41" s="11"/>
+      <x:c r="N41" s="11"/>
+      <x:c r="O41" s="11"/>
+      <x:c r="P41" s="11" t="str">
+        <x:v>Britain</x:v>
+      </x:c>
+      <x:c r="Q41" s="11"/>
+      <x:c r="R41" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S41" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T41" s="11" t="str">
+        <x:v>GB-2022-ELIZABETH-DIES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="11" t="n">
+        <x:v>1912</x:v>
+      </x:c>
+      <x:c r="B42" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C42" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D42" s="11"/>
+      <x:c r="E42" s="11"/>
+      <x:c r="F42" s="11"/>
+      <x:c r="G42" s="11"/>
+      <x:c r="H42" s="11" t="str">
+        <x:v>Republic of China Founded</x:v>
+      </x:c>
+      <x:c r="I42" s="11" t="str">
+        <x:v>The Republic of China was formally established after imperial rule ended.</x:v>
+      </x:c>
+      <x:c r="J42" s="11"/>
+      <x:c r="K42" s="11"/>
+      <x:c r="L42" s="11"/>
+      <x:c r="M42" s="11"/>
+      <x:c r="N42" s="11"/>
+      <x:c r="O42" s="11"/>
+      <x:c r="P42" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q42" s="11"/>
+      <x:c r="R42" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S42" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T42" s="11" t="str">
+        <x:v>CN-1912-ROC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="11" t="n">
+        <x:v>1931</x:v>
+      </x:c>
+      <x:c r="B43" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C43" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D43" s="11"/>
+      <x:c r="E43" s="11"/>
+      <x:c r="F43" s="11"/>
+      <x:c r="G43" s="11"/>
+      <x:c r="H43" s="11" t="str">
+        <x:v>Mukden Incident</x:v>
+      </x:c>
+      <x:c r="I43" s="11" t="str">
+        <x:v>Japan used the incident as a pretext to occupy Manchuria.</x:v>
+      </x:c>
+      <x:c r="J43" s="11"/>
+      <x:c r="K43" s="11"/>
+      <x:c r="L43" s="11"/>
+      <x:c r="M43" s="11"/>
+      <x:c r="N43" s="11"/>
+      <x:c r="O43" s="11"/>
+      <x:c r="P43" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q43" s="11"/>
+      <x:c r="R43" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S43" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T43" s="11" t="str">
+        <x:v>CN-1931-MUKDEN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="11" t="n">
+        <x:v>1945</x:v>
+      </x:c>
+      <x:c r="B44" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C44" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D44" s="11"/>
+      <x:c r="E44" s="11"/>
+      <x:c r="F44" s="11"/>
+      <x:c r="G44" s="11"/>
+      <x:c r="H44" s="11" t="str">
+        <x:v>Japan Formally Surrenders</x:v>
+      </x:c>
+      <x:c r="I44" s="11" t="str">
+        <x:v>Japan’s surrender ended the Second Sino-Japanese War and World War II.</x:v>
+      </x:c>
+      <x:c r="J44" s="11"/>
+      <x:c r="K44" s="11"/>
+      <x:c r="L44" s="11"/>
+      <x:c r="M44" s="11"/>
+      <x:c r="N44" s="11"/>
+      <x:c r="O44" s="11"/>
+      <x:c r="P44" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q44" s="11"/>
+      <x:c r="R44" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S44" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T44" s="11" t="str">
+        <x:v>CN-1945-SURRENDER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="11" t="n">
+        <x:v>1953</x:v>
+      </x:c>
+      <x:c r="B45" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C45" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D45" s="11"/>
+      <x:c r="E45" s="11"/>
+      <x:c r="F45" s="11"/>
+      <x:c r="G45" s="11"/>
+      <x:c r="H45" s="11" t="str">
+        <x:v>First Five-Year Plan Begins</x:v>
+      </x:c>
+      <x:c r="I45" s="11" t="str">
+        <x:v>China launched a state-led industrialization program.</x:v>
+      </x:c>
+      <x:c r="J45" s="11"/>
+      <x:c r="K45" s="11"/>
+      <x:c r="L45" s="11"/>
+      <x:c r="M45" s="11"/>
+      <x:c r="N45" s="11"/>
+      <x:c r="O45" s="11"/>
+      <x:c r="P45" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q45" s="11"/>
+      <x:c r="R45" s="11" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="S45" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T45" s="11" t="str">
+        <x:v>CN-1953-FIVE-YEAR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="11" t="n">
+        <x:v>1958</x:v>
+      </x:c>
+      <x:c r="B46" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C46" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D46" s="11"/>
+      <x:c r="E46" s="11"/>
+      <x:c r="F46" s="11"/>
+      <x:c r="G46" s="11"/>
+      <x:c r="H46" s="11" t="str">
+        <x:v>Great Leap Forward Begins</x:v>
+      </x:c>
+      <x:c r="I46" s="11" t="str">
+        <x:v>The campaign sought rapid industrial and agricultural transformation, with disastrous results.</x:v>
+      </x:c>
+      <x:c r="J46" s="11"/>
+      <x:c r="K46" s="11"/>
+      <x:c r="L46" s="11"/>
+      <x:c r="M46" s="11"/>
+      <x:c r="N46" s="11"/>
+      <x:c r="O46" s="11"/>
+      <x:c r="P46" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q46" s="11"/>
+      <x:c r="R46" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S46" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T46" s="11" t="str">
+        <x:v>CN-1958-GREAT-LEAP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="11" t="n">
+        <x:v>1964</x:v>
+      </x:c>
+      <x:c r="B47" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C47" s="11" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D47" s="11"/>
+      <x:c r="E47" s="11"/>
+      <x:c r="F47" s="11"/>
+      <x:c r="G47" s="11"/>
+      <x:c r="H47" s="11" t="str">
+        <x:v>China Tests Its First Atomic Bomb</x:v>
+      </x:c>
+      <x:c r="I47" s="11" t="str">
+        <x:v>China detonated its first nuclear weapon at Lop Nur.</x:v>
+      </x:c>
+      <x:c r="J47" s="11"/>
+      <x:c r="K47" s="11"/>
+      <x:c r="L47" s="11"/>
+      <x:c r="M47" s="11"/>
+      <x:c r="N47" s="11"/>
+      <x:c r="O47" s="11"/>
+      <x:c r="P47" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q47" s="11"/>
+      <x:c r="R47" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S47" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T47" s="11" t="str">
+        <x:v>CN-1964-NUCLEAR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="11" t="n">
+        <x:v>1976</x:v>
+      </x:c>
+      <x:c r="B48" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C48" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D48" s="11"/>
+      <x:c r="E48" s="11"/>
+      <x:c r="F48" s="11"/>
+      <x:c r="G48" s="11"/>
+      <x:c r="H48" s="11" t="str">
+        <x:v>Mao Zedong Dies</x:v>
+      </x:c>
+      <x:c r="I48" s="11" t="str">
+        <x:v>Mao’s death marked the end of an era in the People’s Republic of China.</x:v>
+      </x:c>
+      <x:c r="J48" s="11"/>
+      <x:c r="K48" s="11"/>
+      <x:c r="L48" s="11"/>
+      <x:c r="M48" s="11"/>
+      <x:c r="N48" s="11"/>
+      <x:c r="O48" s="11"/>
+      <x:c r="P48" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q48" s="11"/>
+      <x:c r="R48" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S48" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T48" s="11" t="str">
+        <x:v>CN-1976-MAO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="11" t="n">
+        <x:v>1979</x:v>
+      </x:c>
+      <x:c r="B49" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C49" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D49" s="11"/>
+      <x:c r="E49" s="11"/>
+      <x:c r="F49" s="11"/>
+      <x:c r="G49" s="11"/>
+      <x:c r="H49" s="11" t="str">
+        <x:v>U.S.–China Diplomatic Relations Established</x:v>
+      </x:c>
+      <x:c r="I49" s="11" t="str">
+        <x:v>The United States and the PRC formally established diplomatic relations.</x:v>
+      </x:c>
+      <x:c r="J49" s="11"/>
+      <x:c r="K49" s="11"/>
+      <x:c r="L49" s="11"/>
+      <x:c r="M49" s="11"/>
+      <x:c r="N49" s="11"/>
+      <x:c r="O49" s="11"/>
+      <x:c r="P49" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q49" s="11"/>
+      <x:c r="R49" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S49" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T49" s="11" t="str">
+        <x:v>CN-1979-DIPLOMACY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="11" t="n">
+        <x:v>1992</x:v>
+      </x:c>
+      <x:c r="B50" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C50" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D50" s="11"/>
+      <x:c r="E50" s="11"/>
+      <x:c r="F50" s="11"/>
+      <x:c r="G50" s="11"/>
+      <x:c r="H50" s="11" t="str">
+        <x:v>Deng Xiaoping’s Southern Tour Begins</x:v>
+      </x:c>
+      <x:c r="I50" s="11" t="str">
+        <x:v>The tour reinforced market-oriented reform and economic opening.</x:v>
+      </x:c>
+      <x:c r="J50" s="11"/>
+      <x:c r="K50" s="11"/>
+      <x:c r="L50" s="11"/>
+      <x:c r="M50" s="11"/>
+      <x:c r="N50" s="11"/>
+      <x:c r="O50" s="11"/>
+      <x:c r="P50" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q50" s="11"/>
+      <x:c r="R50" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S50" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T50" s="11" t="str">
+        <x:v>CN-1992-SOUTHERN-TOUR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="11" t="n">
+        <x:v>1999</x:v>
+      </x:c>
+      <x:c r="B51" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C51" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D51" s="11"/>
+      <x:c r="E51" s="11"/>
+      <x:c r="F51" s="11"/>
+      <x:c r="G51" s="11"/>
+      <x:c r="H51" s="11" t="str">
+        <x:v>Macau Handover</x:v>
+      </x:c>
+      <x:c r="I51" s="11" t="str">
+        <x:v>Portugal transferred sovereignty over Macau to China.</x:v>
+      </x:c>
+      <x:c r="J51" s="11"/>
+      <x:c r="K51" s="11"/>
+      <x:c r="L51" s="11"/>
+      <x:c r="M51" s="11"/>
+      <x:c r="N51" s="11"/>
+      <x:c r="O51" s="11"/>
+      <x:c r="P51" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q51" s="11"/>
+      <x:c r="R51" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S51" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T51" s="11" t="str">
+        <x:v>CN-1999-MACAU</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="11" t="n">
+        <x:v>2003</x:v>
+      </x:c>
+      <x:c r="B52" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C52" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D52" s="11"/>
+      <x:c r="E52" s="11"/>
+      <x:c r="F52" s="11"/>
+      <x:c r="G52" s="11"/>
+      <x:c r="H52" s="11" t="str">
+        <x:v>China Launches First Crewed Spaceflight</x:v>
+      </x:c>
+      <x:c r="I52" s="11" t="str">
+        <x:v>Yang Liwei flew aboard Shenzhou 5.</x:v>
+      </x:c>
+      <x:c r="J52" s="11"/>
+      <x:c r="K52" s="11"/>
+      <x:c r="L52" s="11"/>
+      <x:c r="M52" s="11"/>
+      <x:c r="N52" s="11"/>
+      <x:c r="O52" s="11"/>
+      <x:c r="P52" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q52" s="11"/>
+      <x:c r="R52" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S52" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T52" s="11" t="str">
+        <x:v>CN-2003-SHENZHOU5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="11" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="B53" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C53" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D53" s="11"/>
+      <x:c r="E53" s="11"/>
+      <x:c r="F53" s="11"/>
+      <x:c r="G53" s="11"/>
+      <x:c r="H53" s="11" t="str">
+        <x:v>Tiangong Space Station Completed</x:v>
+      </x:c>
+      <x:c r="I53" s="11" t="str">
+        <x:v>China completed the basic three-module Tiangong station.</x:v>
+      </x:c>
+      <x:c r="J53" s="11"/>
+      <x:c r="K53" s="11"/>
+      <x:c r="L53" s="11"/>
+      <x:c r="M53" s="11"/>
+      <x:c r="N53" s="11"/>
+      <x:c r="O53" s="11"/>
+      <x:c r="P53" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q53" s="11"/>
+      <x:c r="R53" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S53" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T53" s="11" t="str">
+        <x:v>CN-2022-TIANGONG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="11" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="B54" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C54" s="11" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D54" s="11"/>
+      <x:c r="E54" s="11"/>
+      <x:c r="F54" s="11"/>
+      <x:c r="G54" s="11"/>
+      <x:c r="H54" s="11" t="str">
+        <x:v>Chang’e 6 Returns Far-Side Lunar Samples</x:v>
+      </x:c>
+      <x:c r="I54" s="11" t="str">
+        <x:v>Chang’e 6 returned the first samples collected from the Moon’s far side.</x:v>
+      </x:c>
+      <x:c r="J54" s="11"/>
+      <x:c r="K54" s="11"/>
+      <x:c r="L54" s="11"/>
+      <x:c r="M54" s="11"/>
+      <x:c r="N54" s="11"/>
+      <x:c r="O54" s="11"/>
+      <x:c r="P54" s="11" t="str">
+        <x:v>China</x:v>
+      </x:c>
+      <x:c r="Q54" s="11"/>
+      <x:c r="R54" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S54" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T54" s="11" t="str">
+        <x:v>CN-2024-CHANGE6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="11" t="n">
+        <x:v>1918</x:v>
+      </x:c>
+      <x:c r="B55" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C55" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D55" s="11"/>
+      <x:c r="E55" s="11"/>
+      <x:c r="F55" s="11"/>
+      <x:c r="G55" s="11"/>
+      <x:c r="H55" s="11" t="str">
+        <x:v>German Empire Collapses</x:v>
+      </x:c>
+      <x:c r="I55" s="11" t="str">
+        <x:v>Kaiser Wilhelm II abdicated as revolution ended the German Empire.</x:v>
+      </x:c>
+      <x:c r="J55" s="11"/>
+      <x:c r="K55" s="11"/>
+      <x:c r="L55" s="11"/>
+      <x:c r="M55" s="11"/>
+      <x:c r="N55" s="11"/>
+      <x:c r="O55" s="11"/>
+      <x:c r="P55" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q55" s="11"/>
+      <x:c r="R55" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S55" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T55" s="11" t="str">
+        <x:v>DE-1918-EMPIRE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="11" t="n">
+        <x:v>1919</x:v>
+      </x:c>
+      <x:c r="B56" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C56" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D56" s="11"/>
+      <x:c r="E56" s="11"/>
+      <x:c r="F56" s="11"/>
+      <x:c r="G56" s="11"/>
+      <x:c r="H56" s="11" t="str">
+        <x:v>Weimar Constitution Signed</x:v>
+      </x:c>
+      <x:c r="I56" s="11" t="str">
+        <x:v>The constitution established Germany as a parliamentary republic.</x:v>
+      </x:c>
+      <x:c r="J56" s="11"/>
+      <x:c r="K56" s="11"/>
+      <x:c r="L56" s="11"/>
+      <x:c r="M56" s="11"/>
+      <x:c r="N56" s="11"/>
+      <x:c r="O56" s="11"/>
+      <x:c r="P56" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q56" s="11"/>
+      <x:c r="R56" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S56" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T56" s="11" t="str">
+        <x:v>DE-1919-WEIMAR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="11" t="n">
+        <x:v>1923</x:v>
+      </x:c>
+      <x:c r="B57" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C57" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D57" s="11"/>
+      <x:c r="E57" s="11"/>
+      <x:c r="F57" s="11"/>
+      <x:c r="G57" s="11"/>
+      <x:c r="H57" s="11" t="str">
+        <x:v>Beer Hall Putsch Begins</x:v>
+      </x:c>
+      <x:c r="I57" s="11" t="str">
+        <x:v>Hitler and Nazi supporters attempted a failed coup in Munich.</x:v>
+      </x:c>
+      <x:c r="J57" s="11"/>
+      <x:c r="K57" s="11"/>
+      <x:c r="L57" s="11"/>
+      <x:c r="M57" s="11"/>
+      <x:c r="N57" s="11"/>
+      <x:c r="O57" s="11"/>
+      <x:c r="P57" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q57" s="11"/>
+      <x:c r="R57" s="11" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="S57" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T57" s="11" t="str">
+        <x:v>DE-1923-PUTSCH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="11" t="n">
+        <x:v>1933</x:v>
+      </x:c>
+      <x:c r="B58" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C58" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D58" s="11"/>
+      <x:c r="E58" s="11"/>
+      <x:c r="F58" s="11"/>
+      <x:c r="G58" s="11"/>
+      <x:c r="H58" s="11" t="str">
+        <x:v>Hitler Appointed Chancellor</x:v>
+      </x:c>
+      <x:c r="I58" s="11" t="str">
+        <x:v>President Hindenburg appointed Adolf Hitler chancellor.</x:v>
+      </x:c>
+      <x:c r="J58" s="11"/>
+      <x:c r="K58" s="11"/>
+      <x:c r="L58" s="11"/>
+      <x:c r="M58" s="11"/>
+      <x:c r="N58" s="11"/>
+      <x:c r="O58" s="11"/>
+      <x:c r="P58" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q58" s="11"/>
+      <x:c r="R58" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S58" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T58" s="11" t="str">
+        <x:v>DE-1933-HITLER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="11" t="n">
+        <x:v>1938</x:v>
+      </x:c>
+      <x:c r="B59" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C59" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D59" s="11"/>
+      <x:c r="E59" s="11"/>
+      <x:c r="F59" s="11"/>
+      <x:c r="G59" s="11"/>
+      <x:c r="H59" s="11" t="str">
+        <x:v>Kristallnacht</x:v>
+      </x:c>
+      <x:c r="I59" s="11" t="str">
+        <x:v>Nazi authorities and supporters carried out widespread attacks on Jewish communities.</x:v>
+      </x:c>
+      <x:c r="J59" s="11"/>
+      <x:c r="K59" s="11"/>
+      <x:c r="L59" s="11"/>
+      <x:c r="M59" s="11"/>
+      <x:c r="N59" s="11"/>
+      <x:c r="O59" s="11"/>
+      <x:c r="P59" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q59" s="11"/>
+      <x:c r="R59" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S59" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T59" s="11" t="str">
+        <x:v>DE-1938-KRISTALLNACHT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="11" t="n">
+        <x:v>1939</x:v>
+      </x:c>
+      <x:c r="B60" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C60" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D60" s="11"/>
+      <x:c r="E60" s="11"/>
+      <x:c r="F60" s="11"/>
+      <x:c r="G60" s="11"/>
+      <x:c r="H60" s="11" t="str">
+        <x:v>Germany Invades Poland</x:v>
+      </x:c>
+      <x:c r="I60" s="11" t="str">
+        <x:v>The invasion triggered the European phase of World War II.</x:v>
+      </x:c>
+      <x:c r="J60" s="11"/>
+      <x:c r="K60" s="11"/>
+      <x:c r="L60" s="11"/>
+      <x:c r="M60" s="11"/>
+      <x:c r="N60" s="11"/>
+      <x:c r="O60" s="11"/>
+      <x:c r="P60" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q60" s="11"/>
+      <x:c r="R60" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S60" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T60" s="11" t="str">
+        <x:v>DE-1939-POLAND</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="11" t="n">
+        <x:v>1945</x:v>
+      </x:c>
+      <x:c r="B61" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C61" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D61" s="11"/>
+      <x:c r="E61" s="11"/>
+      <x:c r="F61" s="11"/>
+      <x:c r="G61" s="11"/>
+      <x:c r="H61" s="11" t="str">
+        <x:v>Germany Surrenders</x:v>
+      </x:c>
+      <x:c r="I61" s="11" t="str">
+        <x:v>Germany’s unconditional surrender ended the war in Europe.</x:v>
+      </x:c>
+      <x:c r="J61" s="11"/>
+      <x:c r="K61" s="11"/>
+      <x:c r="L61" s="11"/>
+      <x:c r="M61" s="11"/>
+      <x:c r="N61" s="11"/>
+      <x:c r="O61" s="11"/>
+      <x:c r="P61" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q61" s="11"/>
+      <x:c r="R61" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S61" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T61" s="11" t="str">
+        <x:v>DE-1945-SURRENDER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="11" t="n">
+        <x:v>1949</x:v>
+      </x:c>
+      <x:c r="B62" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C62" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D62" s="11"/>
+      <x:c r="E62" s="11"/>
+      <x:c r="F62" s="11"/>
+      <x:c r="G62" s="11"/>
+      <x:c r="H62" s="11" t="str">
+        <x:v>Federal Republic of Germany Founded</x:v>
+      </x:c>
+      <x:c r="I62" s="11" t="str">
+        <x:v>West Germany was established under the Basic Law.</x:v>
+      </x:c>
+      <x:c r="J62" s="11"/>
+      <x:c r="K62" s="11"/>
+      <x:c r="L62" s="11"/>
+      <x:c r="M62" s="11"/>
+      <x:c r="N62" s="11"/>
+      <x:c r="O62" s="11"/>
+      <x:c r="P62" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q62" s="11"/>
+      <x:c r="R62" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S62" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T62" s="11" t="str">
+        <x:v>DE-1949-FRG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="11" t="n">
+        <x:v>1961</x:v>
+      </x:c>
+      <x:c r="B63" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C63" s="11" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D63" s="11"/>
+      <x:c r="E63" s="11"/>
+      <x:c r="F63" s="11"/>
+      <x:c r="G63" s="11"/>
+      <x:c r="H63" s="11" t="str">
+        <x:v>Berlin Wall Construction Begins</x:v>
+      </x:c>
+      <x:c r="I63" s="11" t="str">
+        <x:v>East German authorities sealed the border through Berlin.</x:v>
+      </x:c>
+      <x:c r="J63" s="11"/>
+      <x:c r="K63" s="11"/>
+      <x:c r="L63" s="11"/>
+      <x:c r="M63" s="11"/>
+      <x:c r="N63" s="11"/>
+      <x:c r="O63" s="11"/>
+      <x:c r="P63" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q63" s="11"/>
+      <x:c r="R63" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S63" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T63" s="11" t="str">
+        <x:v>DE-1961-WALL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="11" t="n">
+        <x:v>1963</x:v>
+      </x:c>
+      <x:c r="B64" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C64" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="D64" s="11"/>
+      <x:c r="E64" s="11"/>
+      <x:c r="F64" s="11"/>
+      <x:c r="G64" s="11"/>
+      <x:c r="H64" s="11" t="str">
+        <x:v>Élysée Treaty Signed</x:v>
+      </x:c>
+      <x:c r="I64" s="11" t="str">
+        <x:v>France and West Germany formalized close cooperation.</x:v>
+      </x:c>
+      <x:c r="J64" s="11"/>
+      <x:c r="K64" s="11"/>
+      <x:c r="L64" s="11"/>
+      <x:c r="M64" s="11"/>
+      <x:c r="N64" s="11"/>
+      <x:c r="O64" s="11"/>
+      <x:c r="P64" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q64" s="11"/>
+      <x:c r="R64" s="11" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="S64" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T64" s="11" t="str">
+        <x:v>DE-1963-ELYSEE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="11" t="n">
+        <x:v>1990</x:v>
+      </x:c>
+      <x:c r="B65" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C65" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D65" s="11"/>
+      <x:c r="E65" s="11"/>
+      <x:c r="F65" s="11"/>
+      <x:c r="G65" s="11"/>
+      <x:c r="H65" s="11" t="str">
+        <x:v>German Reunification</x:v>
+      </x:c>
+      <x:c r="I65" s="11" t="str">
+        <x:v>East and West Germany formally reunited.</x:v>
+      </x:c>
+      <x:c r="J65" s="11"/>
+      <x:c r="K65" s="11"/>
+      <x:c r="L65" s="11"/>
+      <x:c r="M65" s="11"/>
+      <x:c r="N65" s="11"/>
+      <x:c r="O65" s="11"/>
+      <x:c r="P65" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q65" s="11"/>
+      <x:c r="R65" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S65" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T65" s="11" t="str">
+        <x:v>DE-1990-REUNIFICATION</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="11" t="n">
+        <x:v>2005</x:v>
+      </x:c>
+      <x:c r="B66" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C66" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="D66" s="11"/>
+      <x:c r="E66" s="11"/>
+      <x:c r="F66" s="11"/>
+      <x:c r="G66" s="11"/>
+      <x:c r="H66" s="11" t="str">
+        <x:v>Angela Merkel Becomes Chancellor</x:v>
+      </x:c>
+      <x:c r="I66" s="11" t="str">
+        <x:v>Merkel became Germany’s first woman chancellor.</x:v>
+      </x:c>
+      <x:c r="J66" s="11"/>
+      <x:c r="K66" s="11"/>
+      <x:c r="L66" s="11"/>
+      <x:c r="M66" s="11"/>
+      <x:c r="N66" s="11"/>
+      <x:c r="O66" s="11"/>
+      <x:c r="P66" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q66" s="11"/>
+      <x:c r="R66" s="11" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="S66" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T66" s="11" t="str">
+        <x:v>DE-2005-MERKEL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="11" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="B67" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C67" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D67" s="11"/>
+      <x:c r="E67" s="11"/>
+      <x:c r="F67" s="11"/>
+      <x:c r="G67" s="11"/>
+      <x:c r="H67" s="11" t="str">
+        <x:v>Germany Ends Nuclear Power Generation</x:v>
+      </x:c>
+      <x:c r="I67" s="11" t="str">
+        <x:v>Germany shut down its final three nuclear power plants.</x:v>
+      </x:c>
+      <x:c r="J67" s="11"/>
+      <x:c r="K67" s="11"/>
+      <x:c r="L67" s="11"/>
+      <x:c r="M67" s="11"/>
+      <x:c r="N67" s="11"/>
+      <x:c r="O67" s="11"/>
+      <x:c r="P67" s="11" t="str">
+        <x:v>Germany</x:v>
+      </x:c>
+      <x:c r="Q67" s="11"/>
+      <x:c r="R67" s="11" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="S67" s="17" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T67" s="11" t="str">
+        <x:v>DE-2023-NUCLEAR</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R942931cbb12f4c95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R272436192c6146e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1077,96 +3177,184 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="11" t="str">
-        <x:v>language_baseline</x:v>
+        <x:v>dataset_name</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
-        <x:v>en</x:v>
+        <x:v>Chrona Modern History Sample</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="11" t="str">
-        <x:v>language_available</x:v>
+        <x:v>dataset_description</x:v>
       </x:c>
       <x:c r="B3" s="11" t="str">
-        <x:v>en,zh-TW,fr,es</x:v>
+        <x:v>Major public events in the United States, Britain, China, and Germany.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="11" t="str">
-        <x:v>primary_groups</x:v>
-      </x:c>
-      <x:c r="B4" s="11" t="str">
-        <x:v>United States</x:v>
-      </x:c>
+      <x:c r="A4" s="11"/>
+      <x:c r="B4" s="11"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="11" t="str">
-        <x:v>group_color.United States</x:v>
+        <x:v>language_baseline</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>#2563EB</x:v>
+        <x:v>en</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="11" t="str">
-        <x:v>group_color.China</x:v>
+        <x:v>language_available</x:v>
       </x:c>
       <x:c r="B6" s="11" t="str">
-        <x:v>#DC2626</x:v>
+        <x:v>en,zh-TW,fr,es,de</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="11" t="str">
-        <x:v>group_color.Ancient Rome</x:v>
-      </x:c>
-      <x:c r="B7" s="11" t="str">
-        <x:v>#7C3AED</x:v>
-      </x:c>
+      <x:c r="A7" s="11"/>
+      <x:c r="B7" s="11"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="11" t="str">
-        <x:v>group_color.Britain</x:v>
+        <x:v>primary_groups</x:v>
       </x:c>
       <x:c r="B8" s="11" t="str">
-        <x:v>#D97706</x:v>
+        <x:v>United States</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="11" t="str">
-        <x:v>group_color.Germany</x:v>
+        <x:v>group_color.United States</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:v>#475569</x:v>
+        <x:v>#2563EB</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="11" t="str">
-        <x:v>never_translate.1</x:v>
+        <x:v>group_color.Britain</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
-        <x:v>Apollo 11</x:v>
+        <x:v>#D97706</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="11" t="str">
-        <x:v>never_translate.2</x:v>
+        <x:v>group_color.China</x:v>
       </x:c>
       <x:c r="B11" s="11" t="str">
-        <x:v>iPhone</x:v>
+        <x:v>#DC2626</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="11" t="str">
-        <x:v>dataset_name</x:v>
+        <x:v>group_color.Germany</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
-        <x:v>Chrona Sample Timeline</x:v>
-      </x:c>
+        <x:v>#475569</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="11" t="str">
+        <x:v>group_color.Ancient Rome</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>#7C3AED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="11"/>
+      <x:c r="B14" s="11"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="11" t="str">
+        <x:v>never_translate.1</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="str">
+        <x:v>Apollo 11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="11" t="str">
+        <x:v>never_translate.2</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="str">
+        <x:v>BBC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="11" t="str">
+        <x:v>never_translate.3</x:v>
+      </x:c>
+      <x:c r="B17" s="11" t="str">
+        <x:v>NHS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="11" t="str">
+        <x:v>never_translate.4</x:v>
+      </x:c>
+      <x:c r="B18" s="11" t="str">
+        <x:v>COVID-19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="11" t="str">
+        <x:v>never_translate.5</x:v>
+      </x:c>
+      <x:c r="B19" s="11" t="str">
+        <x:v>Chang’e 6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="11"/>
+      <x:c r="B20" s="11"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="11"/>
+      <x:c r="B21" s="11"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="11"/>
+      <x:c r="B22" s="11"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="11"/>
+      <x:c r="B23" s="11"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="11"/>
+      <x:c r="B24" s="11"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="11"/>
+      <x:c r="B25" s="11"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="11"/>
+      <x:c r="B26" s="11"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="11"/>
+      <x:c r="B27" s="11"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="11"/>
+      <x:c r="B28" s="11"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="11"/>
+      <x:c r="B29" s="11"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="11"/>
+      <x:c r="B30" s="11"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e0ff29657d04103"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7339159037424f83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>